<commit_message>
fix: mettre a jour les doc plan
</commit_message>
<xml_diff>
--- a/docs/S4/Plan Réel S4.xlsx
+++ b/docs/S4/Plan Réel S4.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E63CF9E-FF82-40D6-BB10-E772DD191D72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46C1840C-301A-4F1E-BCF6-86122E8EA676}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="415" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3214,6 +3214,89 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>10467</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>177940</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1386974</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>186021</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="ZoneTexte 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{42A10078-8BD3-4C16-8B6F-07E8BEEE6F64}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="324478" y="16359973"/>
+          <a:ext cx="6798430" cy="2394564"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="fr-FR" sz="2800">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Les noms des membres du groupe sont indiqués à titre indicatif uniquement. Pour connaître la répartition réelle des tâches, veuillez consulter la fiche de suivi au format Excel.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="fr-FR" sz="1100">
+            <a:solidFill>
+              <a:srgbClr val="FF0000"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -11656,7 +11739,7 @@
       </c>
       <c r="C6" s="32" cm="1">
         <f t="array" aca="1" ref="C6" ca="1">IFERROR(IF(MIN(Jalons435[Début])=0,TODAY(),B11(Jalons435[Début])),TODAY())</f>
-        <v>46193</v>
+        <v>46196</v>
       </c>
       <c r="D6" s="48"/>
       <c r="E6" s="30"/>
@@ -11675,7 +11758,7 @@
       <c r="O6" s="88"/>
       <c r="P6" s="88" t="str">
         <f ca="1">IF(TEXT(P7,"mmmm")=I6,"",TEXT(P7,"mmmm"))</f>
-        <v/>
+        <v>juillet</v>
       </c>
       <c r="Q6" s="88"/>
       <c r="R6" s="88"/>
@@ -11685,7 +11768,7 @@
       <c r="V6" s="88"/>
       <c r="W6" s="88" t="str">
         <f ca="1">IF(OR(TEXT(W7,"mmmm")=P6,TEXT(W7,"mmmm")=I6),"",TEXT(W7,"mmmm"))</f>
-        <v>juillet</v>
+        <v/>
       </c>
       <c r="X6" s="88"/>
       <c r="Y6" s="88"/>
@@ -11760,227 +11843,227 @@
       <c r="H7" s="27"/>
       <c r="I7" s="109">
         <f ca="1">IFERROR(Début_Projet+Incrément_de_défilement,TODAY())</f>
-        <v>46194</v>
+        <v>46197</v>
       </c>
       <c r="J7" s="110">
         <f ca="1">I7+1</f>
-        <v>46195</v>
+        <v>46198</v>
       </c>
       <c r="K7" s="110">
         <f t="shared" ref="K7:AX7" ca="1" si="0">J7+1</f>
-        <v>46196</v>
+        <v>46199</v>
       </c>
       <c r="L7" s="110">
         <f t="shared" ca="1" si="0"/>
-        <v>46197</v>
+        <v>46200</v>
       </c>
       <c r="M7" s="110">
         <f t="shared" ca="1" si="0"/>
-        <v>46198</v>
+        <v>46201</v>
       </c>
       <c r="N7" s="110">
         <f t="shared" ca="1" si="0"/>
-        <v>46199</v>
+        <v>46202</v>
       </c>
       <c r="O7" s="111">
         <f t="shared" ca="1" si="0"/>
-        <v>46200</v>
+        <v>46203</v>
       </c>
       <c r="P7" s="110">
         <f ca="1">O7+1</f>
-        <v>46201</v>
+        <v>46204</v>
       </c>
       <c r="Q7" s="110">
         <f ca="1">P7+1</f>
-        <v>46202</v>
+        <v>46205</v>
       </c>
       <c r="R7" s="110">
         <f t="shared" ca="1" si="0"/>
-        <v>46203</v>
+        <v>46206</v>
       </c>
       <c r="S7" s="110">
         <f t="shared" ca="1" si="0"/>
-        <v>46204</v>
+        <v>46207</v>
       </c>
       <c r="T7" s="110">
         <f t="shared" ca="1" si="0"/>
-        <v>46205</v>
+        <v>46208</v>
       </c>
       <c r="U7" s="110">
         <f t="shared" ca="1" si="0"/>
-        <v>46206</v>
+        <v>46209</v>
       </c>
       <c r="V7" s="111">
         <f t="shared" ca="1" si="0"/>
-        <v>46207</v>
+        <v>46210</v>
       </c>
       <c r="W7" s="110">
         <f ca="1">V7+1</f>
-        <v>46208</v>
+        <v>46211</v>
       </c>
       <c r="X7" s="110">
         <f ca="1">W7+1</f>
-        <v>46209</v>
+        <v>46212</v>
       </c>
       <c r="Y7" s="110">
         <f t="shared" ca="1" si="0"/>
-        <v>46210</v>
+        <v>46213</v>
       </c>
       <c r="Z7" s="110">
         <f t="shared" ca="1" si="0"/>
-        <v>46211</v>
+        <v>46214</v>
       </c>
       <c r="AA7" s="110">
         <f t="shared" ca="1" si="0"/>
-        <v>46212</v>
+        <v>46215</v>
       </c>
       <c r="AB7" s="110">
         <f t="shared" ca="1" si="0"/>
-        <v>46213</v>
+        <v>46216</v>
       </c>
       <c r="AC7" s="111">
         <f t="shared" ca="1" si="0"/>
-        <v>46214</v>
+        <v>46217</v>
       </c>
       <c r="AD7" s="110">
         <f ca="1">AC7+1</f>
-        <v>46215</v>
+        <v>46218</v>
       </c>
       <c r="AE7" s="110">
         <f ca="1">AD7+1</f>
-        <v>46216</v>
+        <v>46219</v>
       </c>
       <c r="AF7" s="110">
         <f t="shared" ca="1" si="0"/>
-        <v>46217</v>
+        <v>46220</v>
       </c>
       <c r="AG7" s="110">
         <f t="shared" ca="1" si="0"/>
-        <v>46218</v>
+        <v>46221</v>
       </c>
       <c r="AH7" s="110">
         <f t="shared" ca="1" si="0"/>
-        <v>46219</v>
+        <v>46222</v>
       </c>
       <c r="AI7" s="110">
         <f t="shared" ca="1" si="0"/>
-        <v>46220</v>
+        <v>46223</v>
       </c>
       <c r="AJ7" s="111">
         <f t="shared" ca="1" si="0"/>
-        <v>46221</v>
+        <v>46224</v>
       </c>
       <c r="AK7" s="110">
         <f ca="1">AJ7+1</f>
-        <v>46222</v>
+        <v>46225</v>
       </c>
       <c r="AL7" s="110">
         <f ca="1">AK7+1</f>
-        <v>46223</v>
+        <v>46226</v>
       </c>
       <c r="AM7" s="110">
         <f t="shared" ca="1" si="0"/>
-        <v>46224</v>
+        <v>46227</v>
       </c>
       <c r="AN7" s="110">
         <f t="shared" ca="1" si="0"/>
-        <v>46225</v>
+        <v>46228</v>
       </c>
       <c r="AO7" s="110">
         <f t="shared" ca="1" si="0"/>
-        <v>46226</v>
+        <v>46229</v>
       </c>
       <c r="AP7" s="110">
         <f t="shared" ca="1" si="0"/>
-        <v>46227</v>
+        <v>46230</v>
       </c>
       <c r="AQ7" s="111">
         <f t="shared" ca="1" si="0"/>
-        <v>46228</v>
+        <v>46231</v>
       </c>
       <c r="AR7" s="110">
         <f ca="1">AQ7+1</f>
-        <v>46229</v>
+        <v>46232</v>
       </c>
       <c r="AS7" s="110">
         <f ca="1">AR7+1</f>
-        <v>46230</v>
+        <v>46233</v>
       </c>
       <c r="AT7" s="110">
         <f t="shared" ca="1" si="0"/>
-        <v>46231</v>
+        <v>46234</v>
       </c>
       <c r="AU7" s="110">
         <f t="shared" ca="1" si="0"/>
-        <v>46232</v>
+        <v>46235</v>
       </c>
       <c r="AV7" s="110">
         <f t="shared" ca="1" si="0"/>
-        <v>46233</v>
+        <v>46236</v>
       </c>
       <c r="AW7" s="110">
         <f t="shared" ca="1" si="0"/>
-        <v>46234</v>
+        <v>46237</v>
       </c>
       <c r="AX7" s="111">
         <f t="shared" ca="1" si="0"/>
-        <v>46235</v>
+        <v>46238</v>
       </c>
       <c r="AY7" s="110">
         <f ca="1">AX7+1</f>
-        <v>46236</v>
+        <v>46239</v>
       </c>
       <c r="AZ7" s="110">
         <f ca="1">AY7+1</f>
-        <v>46237</v>
+        <v>46240</v>
       </c>
       <c r="BA7" s="110">
         <f t="shared" ref="BA7:BE7" ca="1" si="1">AZ7+1</f>
-        <v>46238</v>
+        <v>46241</v>
       </c>
       <c r="BB7" s="110">
         <f t="shared" ca="1" si="1"/>
-        <v>46239</v>
+        <v>46242</v>
       </c>
       <c r="BC7" s="110">
         <f t="shared" ca="1" si="1"/>
-        <v>46240</v>
+        <v>46243</v>
       </c>
       <c r="BD7" s="110">
         <f t="shared" ca="1" si="1"/>
-        <v>46241</v>
+        <v>46244</v>
       </c>
       <c r="BE7" s="111">
         <f t="shared" ca="1" si="1"/>
-        <v>46242</v>
+        <v>46245</v>
       </c>
       <c r="BF7" s="110">
         <f ca="1">BE7+1</f>
-        <v>46243</v>
+        <v>46246</v>
       </c>
       <c r="BG7" s="110">
         <f ca="1">BF7+1</f>
-        <v>46244</v>
+        <v>46247</v>
       </c>
       <c r="BH7" s="110">
         <f t="shared" ref="BH7:BL7" ca="1" si="2">BG7+1</f>
-        <v>46245</v>
+        <v>46248</v>
       </c>
       <c r="BI7" s="110">
         <f t="shared" ca="1" si="2"/>
-        <v>46246</v>
+        <v>46249</v>
       </c>
       <c r="BJ7" s="110">
         <f t="shared" ca="1" si="2"/>
-        <v>46247</v>
+        <v>46250</v>
       </c>
       <c r="BK7" s="110">
         <f t="shared" ca="1" si="2"/>
-        <v>46248</v>
+        <v>46251</v>
       </c>
       <c r="BL7" s="112">
         <f t="shared" ca="1" si="2"/>
-        <v>46249</v>
+        <v>46252</v>
       </c>
       <c r="BM7" s="30"/>
     </row>
@@ -12074,227 +12157,227 @@
       <c r="H9" s="43"/>
       <c r="I9" s="35" t="str">
         <f t="shared" ref="I9:AN9" ca="1" si="3">LEFT(TEXT(I7,"jjj"),1)</f>
-        <v>d</v>
+        <v>m</v>
       </c>
       <c r="J9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>l</v>
+        <v>j</v>
       </c>
       <c r="K9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>m</v>
+        <v>v</v>
       </c>
       <c r="L9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>m</v>
+        <v>s</v>
       </c>
       <c r="M9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>j</v>
+        <v>d</v>
       </c>
       <c r="N9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>v</v>
+        <v>l</v>
       </c>
       <c r="O9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>m</v>
       </c>
       <c r="P9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>m</v>
       </c>
       <c r="Q9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>l</v>
+        <v>j</v>
       </c>
       <c r="R9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>m</v>
+        <v>v</v>
       </c>
       <c r="S9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>m</v>
+        <v>s</v>
       </c>
       <c r="T9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>j</v>
+        <v>d</v>
       </c>
       <c r="U9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>v</v>
+        <v>l</v>
       </c>
       <c r="V9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>m</v>
       </c>
       <c r="W9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>m</v>
       </c>
       <c r="X9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>l</v>
+        <v>j</v>
       </c>
       <c r="Y9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>m</v>
+        <v>v</v>
       </c>
       <c r="Z9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>m</v>
+        <v>s</v>
       </c>
       <c r="AA9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>j</v>
+        <v>d</v>
       </c>
       <c r="AB9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>v</v>
+        <v>l</v>
       </c>
       <c r="AC9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>m</v>
       </c>
       <c r="AD9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>m</v>
       </c>
       <c r="AE9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>l</v>
+        <v>j</v>
       </c>
       <c r="AF9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>m</v>
+        <v>v</v>
       </c>
       <c r="AG9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>m</v>
+        <v>s</v>
       </c>
       <c r="AH9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>j</v>
+        <v>d</v>
       </c>
       <c r="AI9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>v</v>
+        <v>l</v>
       </c>
       <c r="AJ9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>m</v>
       </c>
       <c r="AK9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>m</v>
       </c>
       <c r="AL9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>l</v>
+        <v>j</v>
       </c>
       <c r="AM9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>m</v>
+        <v>v</v>
       </c>
       <c r="AN9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>m</v>
+        <v>s</v>
       </c>
       <c r="AO9" s="35" t="str">
         <f t="shared" ref="AO9:BL9" ca="1" si="4">LEFT(TEXT(AO7,"jjj"),1)</f>
-        <v>j</v>
+        <v>d</v>
       </c>
       <c r="AP9" s="35" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>v</v>
+        <v>l</v>
       </c>
       <c r="AQ9" s="35" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>s</v>
+        <v>m</v>
       </c>
       <c r="AR9" s="35" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>d</v>
+        <v>m</v>
       </c>
       <c r="AS9" s="35" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>l</v>
+        <v>j</v>
       </c>
       <c r="AT9" s="35" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>m</v>
+        <v>v</v>
       </c>
       <c r="AU9" s="35" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>m</v>
+        <v>s</v>
       </c>
       <c r="AV9" s="35" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>j</v>
+        <v>d</v>
       </c>
       <c r="AW9" s="35" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>v</v>
+        <v>l</v>
       </c>
       <c r="AX9" s="35" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>s</v>
+        <v>m</v>
       </c>
       <c r="AY9" s="35" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>d</v>
+        <v>m</v>
       </c>
       <c r="AZ9" s="35" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>l</v>
+        <v>j</v>
       </c>
       <c r="BA9" s="35" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>m</v>
+        <v>v</v>
       </c>
       <c r="BB9" s="35" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>m</v>
+        <v>s</v>
       </c>
       <c r="BC9" s="35" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>j</v>
+        <v>d</v>
       </c>
       <c r="BD9" s="35" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>v</v>
+        <v>l</v>
       </c>
       <c r="BE9" s="35" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>s</v>
+        <v>m</v>
       </c>
       <c r="BF9" s="35" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>d</v>
+        <v>m</v>
       </c>
       <c r="BG9" s="35" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>l</v>
+        <v>j</v>
       </c>
       <c r="BH9" s="35" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>m</v>
+        <v>v</v>
       </c>
       <c r="BI9" s="35" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>m</v>
+        <v>s</v>
       </c>
       <c r="BJ9" s="35" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>j</v>
+        <v>d</v>
       </c>
       <c r="BK9" s="35" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>v</v>
+        <v>l</v>
       </c>
       <c r="BL9" s="35" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>s</v>
+        <v>m</v>
       </c>
       <c r="BM9" s="30"/>
     </row>
@@ -12618,7 +12701,7 @@
       </c>
       <c r="F12" s="21">
         <f ca="1">TODAY()</f>
-        <v>46193</v>
+        <v>46196</v>
       </c>
       <c r="G12" s="22">
         <v>3</v>
@@ -12862,7 +12945,7 @@
       <c r="E13" s="20"/>
       <c r="F13" s="21">
         <f ca="1">TODAY()+5</f>
-        <v>46198</v>
+        <v>46201</v>
       </c>
       <c r="G13" s="22">
         <v>1</v>
@@ -13108,7 +13191,7 @@
       </c>
       <c r="F14" s="21">
         <f ca="1">F12-3</f>
-        <v>46190</v>
+        <v>46193</v>
       </c>
       <c r="G14" s="22">
         <v>10</v>
@@ -13352,7 +13435,7 @@
       <c r="E15" s="20"/>
       <c r="F15" s="21">
         <f ca="1">F12+20</f>
-        <v>46213</v>
+        <v>46216</v>
       </c>
       <c r="G15" s="22">
         <v>1</v>
@@ -13598,7 +13681,7 @@
       </c>
       <c r="F16" s="21">
         <f ca="1">F12+6</f>
-        <v>46199</v>
+        <v>46202</v>
       </c>
       <c r="G16" s="22">
         <v>6</v>
@@ -14081,7 +14164,7 @@
       </c>
       <c r="F18" s="21">
         <f ca="1">F12+6</f>
-        <v>46199</v>
+        <v>46202</v>
       </c>
       <c r="G18" s="22">
         <v>13</v>
@@ -14327,7 +14410,7 @@
       </c>
       <c r="F19" s="21">
         <f ca="1">F18+2</f>
-        <v>46201</v>
+        <v>46204</v>
       </c>
       <c r="G19" s="22">
         <v>9</v>
@@ -14573,7 +14656,7 @@
       </c>
       <c r="F20" s="21">
         <f ca="1">F19+5</f>
-        <v>46206</v>
+        <v>46209</v>
       </c>
       <c r="G20" s="22">
         <v>11</v>
@@ -14817,7 +14900,7 @@
       <c r="E21" s="20"/>
       <c r="F21" s="21">
         <f ca="1">F20+2</f>
-        <v>46208</v>
+        <v>46211</v>
       </c>
       <c r="G21" s="22">
         <v>1</v>
@@ -15059,7 +15142,7 @@
       <c r="E22" s="20"/>
       <c r="F22" s="21">
         <f ca="1">F21+1</f>
-        <v>46209</v>
+        <v>46212</v>
       </c>
       <c r="G22" s="22">
         <v>24</v>
@@ -15540,7 +15623,7 @@
       <c r="E24" s="20"/>
       <c r="F24" s="21">
         <f ca="1">F12+15</f>
-        <v>46208</v>
+        <v>46211</v>
       </c>
       <c r="G24" s="22">
         <v>4</v>
@@ -15784,7 +15867,7 @@
       <c r="E25" s="20"/>
       <c r="F25" s="21">
         <f ca="1">F24+3</f>
-        <v>46211</v>
+        <v>46214</v>
       </c>
       <c r="G25" s="22">
         <v>14</v>
@@ -16028,7 +16111,7 @@
       <c r="E26" s="20"/>
       <c r="F26" s="21">
         <f ca="1">F25+15</f>
-        <v>46226</v>
+        <v>46229</v>
       </c>
       <c r="G26" s="22">
         <v>6</v>
@@ -16272,7 +16355,7 @@
       <c r="E27" s="20"/>
       <c r="F27" s="21">
         <f ca="1">F21+22</f>
-        <v>46230</v>
+        <v>46233</v>
       </c>
       <c r="G27" s="22">
         <v>3</v>
@@ -16516,7 +16599,7 @@
       <c r="E28" s="20"/>
       <c r="F28" s="21">
         <f ca="1">F16</f>
-        <v>46199</v>
+        <v>46202</v>
       </c>
       <c r="G28" s="22">
         <v>19</v>
@@ -16995,7 +17078,7 @@
       <c r="E30" s="20"/>
       <c r="F30" s="21">
         <f ca="1">F27+3</f>
-        <v>46233</v>
+        <v>46236</v>
       </c>
       <c r="G30" s="22">
         <v>15</v>
@@ -17237,7 +17320,7 @@
       <c r="E31" s="20"/>
       <c r="F31" s="21">
         <f ca="1">F30+14</f>
-        <v>46247</v>
+        <v>46250</v>
       </c>
       <c r="G31" s="22">
         <v>5</v>
@@ -17481,7 +17564,7 @@
       <c r="E32" s="20"/>
       <c r="F32" s="21">
         <f ca="1">F31+42</f>
-        <v>46289</v>
+        <v>46292</v>
       </c>
       <c r="G32" s="22">
         <v>1</v>
@@ -18848,7 +18931,7 @@
       </c>
       <c r="C6" s="74" cm="1">
         <f t="array" aca="1" ref="C6" ca="1">IFERROR(IF(MIN(Jalons43524[Début])=0,TODAY(),B11(Jalons43524[Début])),TODAY())</f>
-        <v>46193</v>
+        <v>46196</v>
       </c>
       <c r="D6" s="75"/>
       <c r="E6" s="69"/>
@@ -18867,7 +18950,7 @@
       <c r="O6" s="85"/>
       <c r="P6" s="85" t="str">
         <f ca="1">IF(TEXT(P7,"mmmm")=I6,"",TEXT(P7,"mmmm"))</f>
-        <v/>
+        <v>juillet</v>
       </c>
       <c r="Q6" s="85"/>
       <c r="R6" s="85"/>
@@ -18877,7 +18960,7 @@
       <c r="V6" s="85"/>
       <c r="W6" s="85" t="str">
         <f ca="1">IF(OR(TEXT(W7,"mmmm")=P6,TEXT(W7,"mmmm")=I6),"",TEXT(W7,"mmmm"))</f>
-        <v>juillet</v>
+        <v/>
       </c>
       <c r="X6" s="85"/>
       <c r="Y6" s="85"/>
@@ -18951,227 +19034,227 @@
       <c r="H7" s="77"/>
       <c r="I7" s="116">
         <f ca="1">IFERROR(Début_Projet+Incrément_de_défilement,TODAY())</f>
-        <v>46194</v>
+        <v>46197</v>
       </c>
       <c r="J7" s="117">
         <f ca="1">I7+1</f>
-        <v>46195</v>
+        <v>46198</v>
       </c>
       <c r="K7" s="117">
         <f t="shared" ref="K7:AX7" ca="1" si="0">J7+1</f>
-        <v>46196</v>
+        <v>46199</v>
       </c>
       <c r="L7" s="117">
         <f t="shared" ca="1" si="0"/>
-        <v>46197</v>
+        <v>46200</v>
       </c>
       <c r="M7" s="117">
         <f t="shared" ca="1" si="0"/>
-        <v>46198</v>
+        <v>46201</v>
       </c>
       <c r="N7" s="117">
         <f t="shared" ca="1" si="0"/>
-        <v>46199</v>
+        <v>46202</v>
       </c>
       <c r="O7" s="118">
         <f t="shared" ca="1" si="0"/>
-        <v>46200</v>
+        <v>46203</v>
       </c>
       <c r="P7" s="117">
         <f ca="1">O7+1</f>
-        <v>46201</v>
+        <v>46204</v>
       </c>
       <c r="Q7" s="117">
         <f ca="1">P7+1</f>
-        <v>46202</v>
+        <v>46205</v>
       </c>
       <c r="R7" s="117">
         <f t="shared" ca="1" si="0"/>
-        <v>46203</v>
+        <v>46206</v>
       </c>
       <c r="S7" s="117">
         <f t="shared" ca="1" si="0"/>
-        <v>46204</v>
+        <v>46207</v>
       </c>
       <c r="T7" s="117">
         <f t="shared" ca="1" si="0"/>
-        <v>46205</v>
+        <v>46208</v>
       </c>
       <c r="U7" s="117">
         <f t="shared" ca="1" si="0"/>
-        <v>46206</v>
+        <v>46209</v>
       </c>
       <c r="V7" s="118">
         <f t="shared" ca="1" si="0"/>
-        <v>46207</v>
+        <v>46210</v>
       </c>
       <c r="W7" s="117">
         <f ca="1">V7+1</f>
-        <v>46208</v>
+        <v>46211</v>
       </c>
       <c r="X7" s="117">
         <f ca="1">W7+1</f>
-        <v>46209</v>
+        <v>46212</v>
       </c>
       <c r="Y7" s="117">
         <f t="shared" ca="1" si="0"/>
-        <v>46210</v>
+        <v>46213</v>
       </c>
       <c r="Z7" s="117">
         <f t="shared" ca="1" si="0"/>
-        <v>46211</v>
+        <v>46214</v>
       </c>
       <c r="AA7" s="117">
         <f t="shared" ca="1" si="0"/>
-        <v>46212</v>
+        <v>46215</v>
       </c>
       <c r="AB7" s="117">
         <f t="shared" ca="1" si="0"/>
-        <v>46213</v>
+        <v>46216</v>
       </c>
       <c r="AC7" s="118">
         <f t="shared" ca="1" si="0"/>
-        <v>46214</v>
+        <v>46217</v>
       </c>
       <c r="AD7" s="117">
         <f ca="1">AC7+1</f>
-        <v>46215</v>
+        <v>46218</v>
       </c>
       <c r="AE7" s="117">
         <f ca="1">AD7+1</f>
-        <v>46216</v>
+        <v>46219</v>
       </c>
       <c r="AF7" s="117">
         <f t="shared" ca="1" si="0"/>
-        <v>46217</v>
+        <v>46220</v>
       </c>
       <c r="AG7" s="117">
         <f t="shared" ca="1" si="0"/>
-        <v>46218</v>
+        <v>46221</v>
       </c>
       <c r="AH7" s="117">
         <f t="shared" ca="1" si="0"/>
-        <v>46219</v>
+        <v>46222</v>
       </c>
       <c r="AI7" s="117">
         <f t="shared" ca="1" si="0"/>
-        <v>46220</v>
+        <v>46223</v>
       </c>
       <c r="AJ7" s="118">
         <f t="shared" ca="1" si="0"/>
-        <v>46221</v>
+        <v>46224</v>
       </c>
       <c r="AK7" s="117">
         <f ca="1">AJ7+1</f>
-        <v>46222</v>
+        <v>46225</v>
       </c>
       <c r="AL7" s="117">
         <f ca="1">AK7+1</f>
-        <v>46223</v>
+        <v>46226</v>
       </c>
       <c r="AM7" s="117">
         <f t="shared" ca="1" si="0"/>
-        <v>46224</v>
+        <v>46227</v>
       </c>
       <c r="AN7" s="117">
         <f t="shared" ca="1" si="0"/>
-        <v>46225</v>
+        <v>46228</v>
       </c>
       <c r="AO7" s="117">
         <f t="shared" ca="1" si="0"/>
-        <v>46226</v>
+        <v>46229</v>
       </c>
       <c r="AP7" s="117">
         <f t="shared" ca="1" si="0"/>
-        <v>46227</v>
+        <v>46230</v>
       </c>
       <c r="AQ7" s="118">
         <f t="shared" ca="1" si="0"/>
-        <v>46228</v>
+        <v>46231</v>
       </c>
       <c r="AR7" s="117">
         <f ca="1">AQ7+1</f>
-        <v>46229</v>
+        <v>46232</v>
       </c>
       <c r="AS7" s="117">
         <f ca="1">AR7+1</f>
-        <v>46230</v>
+        <v>46233</v>
       </c>
       <c r="AT7" s="117">
         <f t="shared" ca="1" si="0"/>
-        <v>46231</v>
+        <v>46234</v>
       </c>
       <c r="AU7" s="117">
         <f t="shared" ca="1" si="0"/>
-        <v>46232</v>
+        <v>46235</v>
       </c>
       <c r="AV7" s="117">
         <f t="shared" ca="1" si="0"/>
-        <v>46233</v>
+        <v>46236</v>
       </c>
       <c r="AW7" s="117">
         <f t="shared" ca="1" si="0"/>
-        <v>46234</v>
+        <v>46237</v>
       </c>
       <c r="AX7" s="118">
         <f t="shared" ca="1" si="0"/>
-        <v>46235</v>
+        <v>46238</v>
       </c>
       <c r="AY7" s="117">
         <f ca="1">AX7+1</f>
-        <v>46236</v>
+        <v>46239</v>
       </c>
       <c r="AZ7" s="117">
         <f ca="1">AY7+1</f>
-        <v>46237</v>
+        <v>46240</v>
       </c>
       <c r="BA7" s="117">
         <f t="shared" ref="BA7:BE7" ca="1" si="1">AZ7+1</f>
-        <v>46238</v>
+        <v>46241</v>
       </c>
       <c r="BB7" s="117">
         <f t="shared" ca="1" si="1"/>
-        <v>46239</v>
+        <v>46242</v>
       </c>
       <c r="BC7" s="117">
         <f t="shared" ca="1" si="1"/>
-        <v>46240</v>
+        <v>46243</v>
       </c>
       <c r="BD7" s="117">
         <f t="shared" ca="1" si="1"/>
-        <v>46241</v>
+        <v>46244</v>
       </c>
       <c r="BE7" s="118">
         <f t="shared" ca="1" si="1"/>
-        <v>46242</v>
+        <v>46245</v>
       </c>
       <c r="BF7" s="117">
         <f ca="1">BE7+1</f>
-        <v>46243</v>
+        <v>46246</v>
       </c>
       <c r="BG7" s="117">
         <f ca="1">BF7+1</f>
-        <v>46244</v>
+        <v>46247</v>
       </c>
       <c r="BH7" s="117">
         <f t="shared" ref="BH7:BL7" ca="1" si="2">BG7+1</f>
-        <v>46245</v>
+        <v>46248</v>
       </c>
       <c r="BI7" s="117">
         <f t="shared" ca="1" si="2"/>
-        <v>46246</v>
+        <v>46249</v>
       </c>
       <c r="BJ7" s="117">
         <f t="shared" ca="1" si="2"/>
-        <v>46247</v>
+        <v>46250</v>
       </c>
       <c r="BK7" s="117">
         <f t="shared" ca="1" si="2"/>
-        <v>46248</v>
+        <v>46251</v>
       </c>
       <c r="BL7" s="118">
         <f t="shared" ca="1" si="2"/>
-        <v>46249</v>
+        <v>46252</v>
       </c>
     </row>
     <row r="8" spans="1:68" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -19263,227 +19346,227 @@
       <c r="H9" s="82"/>
       <c r="I9" s="91" t="str">
         <f t="shared" ref="I9:AN9" ca="1" si="3">LEFT(TEXT(I7,"jjj"),1)</f>
-        <v>d</v>
+        <v>m</v>
       </c>
       <c r="J9" s="91" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>l</v>
+        <v>j</v>
       </c>
       <c r="K9" s="91" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>m</v>
+        <v>v</v>
       </c>
       <c r="L9" s="91" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>m</v>
+        <v>s</v>
       </c>
       <c r="M9" s="91" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>j</v>
+        <v>d</v>
       </c>
       <c r="N9" s="91" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>v</v>
+        <v>l</v>
       </c>
       <c r="O9" s="91" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>m</v>
       </c>
       <c r="P9" s="91" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>m</v>
       </c>
       <c r="Q9" s="91" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>l</v>
+        <v>j</v>
       </c>
       <c r="R9" s="91" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>m</v>
+        <v>v</v>
       </c>
       <c r="S9" s="91" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>m</v>
+        <v>s</v>
       </c>
       <c r="T9" s="91" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>j</v>
+        <v>d</v>
       </c>
       <c r="U9" s="91" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>v</v>
+        <v>l</v>
       </c>
       <c r="V9" s="91" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>m</v>
       </c>
       <c r="W9" s="91" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>m</v>
       </c>
       <c r="X9" s="91" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>l</v>
+        <v>j</v>
       </c>
       <c r="Y9" s="91" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>m</v>
+        <v>v</v>
       </c>
       <c r="Z9" s="91" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>m</v>
+        <v>s</v>
       </c>
       <c r="AA9" s="91" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>j</v>
+        <v>d</v>
       </c>
       <c r="AB9" s="91" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>v</v>
+        <v>l</v>
       </c>
       <c r="AC9" s="91" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>m</v>
       </c>
       <c r="AD9" s="91" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>m</v>
       </c>
       <c r="AE9" s="91" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>l</v>
+        <v>j</v>
       </c>
       <c r="AF9" s="91" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>m</v>
+        <v>v</v>
       </c>
       <c r="AG9" s="91" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>m</v>
+        <v>s</v>
       </c>
       <c r="AH9" s="91" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>j</v>
+        <v>d</v>
       </c>
       <c r="AI9" s="91" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>v</v>
+        <v>l</v>
       </c>
       <c r="AJ9" s="91" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>m</v>
       </c>
       <c r="AK9" s="91" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>m</v>
       </c>
       <c r="AL9" s="91" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>l</v>
+        <v>j</v>
       </c>
       <c r="AM9" s="91" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>m</v>
+        <v>v</v>
       </c>
       <c r="AN9" s="91" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>m</v>
+        <v>s</v>
       </c>
       <c r="AO9" s="91" t="str">
         <f t="shared" ref="AO9:BL9" ca="1" si="4">LEFT(TEXT(AO7,"jjj"),1)</f>
-        <v>j</v>
+        <v>d</v>
       </c>
       <c r="AP9" s="91" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>v</v>
+        <v>l</v>
       </c>
       <c r="AQ9" s="91" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>s</v>
+        <v>m</v>
       </c>
       <c r="AR9" s="91" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>d</v>
+        <v>m</v>
       </c>
       <c r="AS9" s="91" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>l</v>
+        <v>j</v>
       </c>
       <c r="AT9" s="91" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>m</v>
+        <v>v</v>
       </c>
       <c r="AU9" s="91" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>m</v>
+        <v>s</v>
       </c>
       <c r="AV9" s="91" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>j</v>
+        <v>d</v>
       </c>
       <c r="AW9" s="91" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>v</v>
+        <v>l</v>
       </c>
       <c r="AX9" s="91" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>s</v>
+        <v>m</v>
       </c>
       <c r="AY9" s="91" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>d</v>
+        <v>m</v>
       </c>
       <c r="AZ9" s="91" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>l</v>
+        <v>j</v>
       </c>
       <c r="BA9" s="91" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>m</v>
+        <v>v</v>
       </c>
       <c r="BB9" s="91" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>m</v>
+        <v>s</v>
       </c>
       <c r="BC9" s="91" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>j</v>
+        <v>d</v>
       </c>
       <c r="BD9" s="91" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>v</v>
+        <v>l</v>
       </c>
       <c r="BE9" s="91" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>s</v>
+        <v>m</v>
       </c>
       <c r="BF9" s="91" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>d</v>
+        <v>m</v>
       </c>
       <c r="BG9" s="91" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>l</v>
+        <v>j</v>
       </c>
       <c r="BH9" s="91" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>m</v>
+        <v>v</v>
       </c>
       <c r="BI9" s="91" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>m</v>
+        <v>s</v>
       </c>
       <c r="BJ9" s="91" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>j</v>
+        <v>d</v>
       </c>
       <c r="BK9" s="91" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>v</v>
+        <v>l</v>
       </c>
       <c r="BL9" s="91" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>s</v>
+        <v>m</v>
       </c>
     </row>
     <row r="10" spans="1:68" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
@@ -19803,7 +19886,7 @@
       </c>
       <c r="F12" s="56">
         <f ca="1">TODAY()</f>
-        <v>46193</v>
+        <v>46196</v>
       </c>
       <c r="G12" s="57">
         <v>3</v>
@@ -20046,7 +20129,7 @@
       <c r="E13" s="55"/>
       <c r="F13" s="56">
         <f ca="1">TODAY()+5</f>
-        <v>46198</v>
+        <v>46201</v>
       </c>
       <c r="G13" s="57">
         <v>1</v>
@@ -20291,7 +20374,7 @@
       </c>
       <c r="F14" s="56">
         <f ca="1">F12-3</f>
-        <v>46190</v>
+        <v>46193</v>
       </c>
       <c r="G14" s="57">
         <v>10</v>
@@ -20534,7 +20617,7 @@
       <c r="E15" s="55"/>
       <c r="F15" s="56">
         <f ca="1">F12+20</f>
-        <v>46213</v>
+        <v>46216</v>
       </c>
       <c r="G15" s="57">
         <v>1</v>
@@ -20779,7 +20862,7 @@
       </c>
       <c r="F16" s="56">
         <f ca="1">F12+6</f>
-        <v>46199</v>
+        <v>46202</v>
       </c>
       <c r="G16" s="57">
         <v>6</v>
@@ -21260,7 +21343,7 @@
       </c>
       <c r="F18" s="56">
         <f ca="1">F12+6</f>
-        <v>46199</v>
+        <v>46202</v>
       </c>
       <c r="G18" s="57">
         <v>13</v>
@@ -21505,7 +21588,7 @@
       </c>
       <c r="F19" s="56">
         <f ca="1">F18+2</f>
-        <v>46201</v>
+        <v>46204</v>
       </c>
       <c r="G19" s="57">
         <v>9</v>
@@ -21750,7 +21833,7 @@
       </c>
       <c r="F20" s="56">
         <f ca="1">F19+5</f>
-        <v>46206</v>
+        <v>46209</v>
       </c>
       <c r="G20" s="57">
         <v>11</v>
@@ -21993,7 +22076,7 @@
       <c r="E21" s="55"/>
       <c r="F21" s="56">
         <f ca="1">F20+2</f>
-        <v>46208</v>
+        <v>46211</v>
       </c>
       <c r="G21" s="57">
         <v>1</v>
@@ -22234,7 +22317,7 @@
       <c r="E22" s="55"/>
       <c r="F22" s="56">
         <f ca="1">F21+1</f>
-        <v>46209</v>
+        <v>46212</v>
       </c>
       <c r="G22" s="57">
         <v>24</v>
@@ -22713,7 +22796,7 @@
       <c r="E24" s="55"/>
       <c r="F24" s="56">
         <f ca="1">F12+15</f>
-        <v>46208</v>
+        <v>46211</v>
       </c>
       <c r="G24" s="57">
         <v>4</v>
@@ -22956,7 +23039,7 @@
       <c r="E25" s="55"/>
       <c r="F25" s="56">
         <f ca="1">F24+3</f>
-        <v>46211</v>
+        <v>46214</v>
       </c>
       <c r="G25" s="57">
         <v>14</v>
@@ -23199,7 +23282,7 @@
       <c r="E26" s="55"/>
       <c r="F26" s="56">
         <f ca="1">F25+15</f>
-        <v>46226</v>
+        <v>46229</v>
       </c>
       <c r="G26" s="57">
         <v>6</v>
@@ -23442,7 +23525,7 @@
       <c r="E27" s="55"/>
       <c r="F27" s="56">
         <f ca="1">F21+22</f>
-        <v>46230</v>
+        <v>46233</v>
       </c>
       <c r="G27" s="57">
         <v>3</v>
@@ -23685,7 +23768,7 @@
       <c r="E28" s="55"/>
       <c r="F28" s="56">
         <f ca="1">F16</f>
-        <v>46199</v>
+        <v>46202</v>
       </c>
       <c r="G28" s="57">
         <v>19</v>
@@ -24162,7 +24245,7 @@
       <c r="E30" s="55"/>
       <c r="F30" s="56">
         <f ca="1">F27+3</f>
-        <v>46233</v>
+        <v>46236</v>
       </c>
       <c r="G30" s="57">
         <v>15</v>
@@ -24403,7 +24486,7 @@
       <c r="E31" s="55"/>
       <c r="F31" s="56">
         <f ca="1">F30+14</f>
-        <v>46247</v>
+        <v>46250</v>
       </c>
       <c r="G31" s="57">
         <v>5</v>
@@ -24646,7 +24729,7 @@
       <c r="E32" s="55"/>
       <c r="F32" s="56">
         <f ca="1">F31+42</f>
-        <v>46289</v>
+        <v>46292</v>
       </c>
       <c r="G32" s="57">
         <v>1</v>
@@ -25841,15 +25924,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
@@ -25866,6 +25940,15 @@
     <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -26145,14 +26228,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{39060724-9CA2-4290-8A0C-B53624A594E7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA4BA2A8-DB97-40F9-8DB6-154C09C7467C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -26160,6 +26235,14 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
     <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
     <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{39060724-9CA2-4290-8A0C-B53624A594E7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>